<commit_message>
Block styles and footer progress
Automated migration updates generated by Experience Modernization Agent.

Changed files (13):
- blocks/cards-featured/cards-featured.css
- blocks/cards-insights/cards-insights.css
- blocks/carousel/carousel.css
- blocks/carousel/carousel.js
- blocks/footer/footer.css
- blocks/footer/footer.js
- footer.plain.html
- tools/importer/import-services-page.bundle.js
- tools/importer/import-services-page.js
- tools/importer/page-templates.json
- tools/importer/parsers/carousel.js
- tools/importer/reports/import-services-page.report.xlsx
- tools/importer/reports/services/family-office-services.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-services-page.report.xlsx
+++ b/tools/importer/reports/import-services-page.report.xlsx
@@ -40,7 +40,7 @@
     <t>services/family-office-services.report.json</t>
   </si>
   <si>
-    <t>["hero-split","columns-featured","columns-featured","columns-highlight","quote","stats","carousel","cards-featured","cards-insights"]</t>
+    <t>["hero-split","columns-featured","columns-featured","columns-highlight","quote","stats","carousel-contacts","cards-featured","cards-insights"]</t>
   </si>
   <si>
     <t>services/family-office-services</t>
@@ -52,7 +52,7 @@
     <t>services-page</t>
   </si>
   <si>
-    <t>2026-05-01T18:58:44.209Z</t>
+    <t>2026-05-02T01:56:19.067Z</t>
   </si>
   <si>
     <t>Family Office Services | Accounting &amp; Advisory Services</t>

</xml_diff>